<commit_message>
Resíduo de Cox-Snell consertados
</commit_message>
<xml_diff>
--- a/arquivos/Análise dos Modelos e Resíduos.xlsx
+++ b/arquivos/Análise dos Modelos e Resíduos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Documents\UnB\Análise de Sobrevivência\Turnover-Sobrevivencia\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3256A7-3609-4663-BAD6-E69168370492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45479DBC-BCED-41B5-9DA1-4DD351FD5295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{4990E75E-E9B6-48C4-892A-4CD4323C3EFF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{4990E75E-E9B6-48C4-892A-4CD4323C3EFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Rank Medidas" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Modelos locação e escala feitos
</commit_message>
<xml_diff>
--- a/arquivos/Análise dos Modelos e Resíduos.xlsx
+++ b/arquivos/Análise dos Modelos e Resíduos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Documents\UnB\Análise de Sobrevivência\Turnover-Sobrevivencia\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082BDA81-8962-4526-8574-9D4760455428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB0CFA9-0E4C-4AD7-8C36-D40CAE56ADCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{4990E75E-E9B6-48C4-892A-4CD4323C3EFF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="8" xr2:uid="{4990E75E-E9B6-48C4-892A-4CD4323C3EFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Rank Medidas" sheetId="1" r:id="rId1"/>
@@ -291,7 +291,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="33">
   <si>
     <t>Exponencial</t>
   </si>
@@ -385,6 +385,12 @@
   <si>
     <t>Logística</t>
   </si>
+  <si>
+    <t>Com 7 variáveis</t>
+  </si>
+  <si>
+    <t>Com 8 variáveis</t>
+  </si>
 </sst>
 </file>
 
@@ -393,7 +399,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -426,6 +432,22 @@
       <color rgb="FF000000"/>
       <name val="Lucida Console"/>
       <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -460,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -475,6 +497,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -795,6 +823,631 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10017900" y="0"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>593912</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>33617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>20171</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>186017</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{208D4ECE-3891-2281-8EE0-413B09487D27}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4224618" y="33617"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>26734</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>4323</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>58111</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>156723</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagem 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5C5F134-5AA8-B1EE-AEA5-C6FDE6A62315}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9103499" y="4323"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BEA4B830-43D1-A392-F309-4D172433284B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3952875" y="0"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>226200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>226200</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagem 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9EC3F288-5F05-0FCA-3E7E-405B9F892C06}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8151000" y="0"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>503464</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>502702</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6CBAE65C-C7FE-5055-2EB1-889D11869F30}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9075964" y="0"/>
+          <a:ext cx="4285488" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>136392</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>135630</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagem 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26686C35-5EED-B3A3-F261-89B9CC7E9F4C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4422642" y="0"/>
+          <a:ext cx="4285488" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D3C60C0-4535-6A44-3216-59906E3939BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4267200" y="0"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>188100</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>188100</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagem 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{92E6A593-29C7-17B6-1170-F79D67AD7D49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8722500" y="0"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{84652ADC-C2A2-246B-7026-3D4A02A4393F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8734425" y="200025"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>7125</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>7125</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>7125</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>159525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagem 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B2B82315-4AEF-3486-FEA0-728664FF7BFA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4274325" y="197625"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Imagem 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{88A4C1A3-0F71-3301-CD6B-07D591384DB1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8534400" y="3943350"/>
+          <a:ext cx="4267200" cy="3200400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>597675</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>7125</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>597675</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>159525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Imagem 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{88CA2B72-DF2E-9FA6-D3AF-0E87FECCC382}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4255275" y="3893325"/>
           <a:ext cx="4267200" cy="3200400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2059,7 +2712,8 @@
   </sheetData>
   <autoFilter ref="A1:E15" xr:uid="{3DACB37D-A5A3-4389-BA22-D76D602171D1}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <legacyDrawing r:id="rId1"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2262,7 +2916,8 @@
   </sheetData>
   <autoFilter ref="A1:F15" xr:uid="{22565C3B-161B-407D-94A8-41234554A020}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <legacyDrawing r:id="rId1"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2464,7 +3119,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <legacyDrawing r:id="rId1"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2671,16 +3327,17 @@
   </sheetData>
   <autoFilter ref="A1:F15" xr:uid="{05B6B6E6-D7BC-4DCC-8A98-370E342E72EC}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <legacyDrawing r:id="rId1"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{548AB32E-D3F8-4E78-B467-F054DF81A492}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -2696,13 +3353,29 @@
       <c r="E1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H1" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -2720,7 +3393,7 @@
         <v>age  +</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -2738,7 +3411,7 @@
         <v>industry  +</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -2756,7 +3429,7 @@
         <v>profession  +</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -2774,7 +3447,7 @@
         <v>traffic  +</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>14</v>
       </c>
@@ -2789,12 +3462,12 @@
         <v>coach  +</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2812,7 +3485,7 @@
         <v>greywage  +</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -2821,17 +3494,17 @@
         <v>way  +</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -2849,7 +3522,7 @@
         <v>selfcontrol  +</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -2867,12 +3540,35 @@
         <v>anxiety  ,</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>7</v>
       </c>
     </row>
+    <row r="20" spans="8:21" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="H20" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="10"/>
+      <c r="U20" s="10"/>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="H1:U1"/>
+    <mergeCell ref="H20:U20"/>
+  </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Teste de independencia de V cramer
</commit_message>
<xml_diff>
--- a/arquivos/Análise dos Modelos e Resíduos.xlsx
+++ b/arquivos/Análise dos Modelos e Resíduos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Documents\UnB\Análise de Sobrevivência\Turnover-Sobrevivencia\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB0CFA9-0E4C-4AD7-8C36-D40CAE56ADCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BD2DE7-0640-427D-809C-EA36D7D960AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="8" xr2:uid="{4990E75E-E9B6-48C4-892A-4CD4323C3EFF}"/>
+    <workbookView xWindow="10140" yWindow="0" windowWidth="10455" windowHeight="10905" firstSheet="3" activeTab="9" xr2:uid="{4990E75E-E9B6-48C4-892A-4CD4323C3EFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Rank Medidas" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="Extremo" sheetId="7" r:id="rId7"/>
     <sheet name="Gaussiana" sheetId="8" r:id="rId8"/>
     <sheet name="logística" sheetId="9" r:id="rId9"/>
+    <sheet name="Planilha1" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Exponencial!$A$1:$E$15</definedName>
@@ -259,7 +260,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
@@ -291,7 +292,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="41">
   <si>
     <t>Exponencial</t>
   </si>
@@ -391,6 +392,30 @@
   <si>
     <t>Com 8 variáveis</t>
   </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Industry</t>
+  </si>
+  <si>
+    <t>Profession</t>
+  </si>
+  <si>
+    <t>Traffic</t>
+  </si>
+  <si>
+    <t>Coach</t>
+  </si>
+  <si>
+    <t>Head_Gender</t>
+  </si>
+  <si>
+    <t>Greywage</t>
+  </si>
+  <si>
+    <t>Way</t>
+  </si>
 </sst>
 </file>
 
@@ -399,7 +424,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -449,6 +474,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -482,7 +515,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -497,12 +530,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1967,6 +2001,466 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1DBB185-36E5-4149-88BE-A59B3EF8D5A3}">
+  <dimension ref="A1:Q9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="10" width="60.28515625" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="61.42578125" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="13" max="15" width="9.140625" customWidth="1"/>
+    <col min="16" max="16" width="65.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O1" t="s">
+        <v>38</v>
+      </c>
+      <c r="P1" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7">
+        <v>0.1863235</v>
+      </c>
+      <c r="D2" s="7">
+        <v>0.49558930000000001</v>
+      </c>
+      <c r="E2" s="7">
+        <v>0.1568532</v>
+      </c>
+      <c r="J2" t="str">
+        <f>_xlfn.CONCAT("CramerV( turnover_limpo$",$B$1,",","turnover_limpo$",A2, ")")</f>
+        <v>CramerV( turnover_limpo$gender  ,turnover_limpo$gender  )</v>
+      </c>
+      <c r="K2" t="str">
+        <f>_xlfn.CONCAT("CramerV( turnover_limpo$",$C$1,",","turnover_limpo$",A2, ")")</f>
+        <v>CramerV( turnover_limpo$industry  ,turnover_limpo$gender  )</v>
+      </c>
+      <c r="L2" t="str">
+        <f>_xlfn.CONCAT("CramerV( turnover_limpo$",$D$1,",","turnover_limpo$",A2, ")")</f>
+        <v>CramerV( turnover_limpo$profession  ,turnover_limpo$gender  )</v>
+      </c>
+      <c r="M2" t="str">
+        <f>_xlfn.CONCAT("CramerV( turnover_limpo$",$E$1,",","turnover_limpo$",A2, ")")</f>
+        <v>CramerV( turnover_limpo$traffic  ,turnover_limpo$gender  )</v>
+      </c>
+      <c r="N2" t="str">
+        <f>_xlfn.CONCAT("CramerV( turnover_limpo$",$F$1,",","turnover_limpo$",A2, ")")</f>
+        <v>CramerV( turnover_limpo$coach  ,turnover_limpo$gender  )</v>
+      </c>
+      <c r="O2" t="str">
+        <f>_xlfn.CONCAT("CramerV( turnover_limpo$",$G$1,",","turnover_limpo$",A2, ")")</f>
+        <v>CramerV( turnover_limpo$head_gender  ,turnover_limpo$gender  )</v>
+      </c>
+      <c r="P2" t="str">
+        <f>_xlfn.CONCAT("CramerV( turnover_limpo$",$H$1,",","turnover_limpo$",A2, ")")</f>
+        <v>CramerV( turnover_limpo$greywage  ,turnover_limpo$gender  )</v>
+      </c>
+      <c r="Q2" t="str">
+        <f>_xlfn.CONCAT("CramerV( turnover_limpo$",$I$1,",","turnover_limpo$",A2, ")")</f>
+        <v>CramerV( turnover_limpo$way  ,turnover_limpo$gender  )</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="7">
+        <v>0.1863235</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" s="7">
+        <v>0.23831939999999999</v>
+      </c>
+      <c r="E3" s="7">
+        <v>0.17210690000000001</v>
+      </c>
+      <c r="J3" t="str">
+        <f t="shared" ref="J3:J10" si="0">_xlfn.CONCAT("CramerV( turnover_limpo$",$B$1,",","turnover_limpo$",A3, ")")</f>
+        <v>CramerV( turnover_limpo$gender  ,turnover_limpo$industry  )</v>
+      </c>
+      <c r="K3" t="str">
+        <f t="shared" ref="K3:K9" si="1">_xlfn.CONCAT("CramerV( turnover_limpo$",$C$1,",","turnover_limpo$",A3, ")")</f>
+        <v>CramerV( turnover_limpo$industry  ,turnover_limpo$industry  )</v>
+      </c>
+      <c r="L3" t="str">
+        <f t="shared" ref="L3:L9" si="2">_xlfn.CONCAT("CramerV( turnover_limpo$",$D$1,",","turnover_limpo$",A3, ")")</f>
+        <v>CramerV( turnover_limpo$profession  ,turnover_limpo$industry  )</v>
+      </c>
+      <c r="M3" t="str">
+        <f t="shared" ref="M3:M9" si="3">_xlfn.CONCAT("CramerV( turnover_limpo$",$E$1,",","turnover_limpo$",A3, ")")</f>
+        <v>CramerV( turnover_limpo$traffic  ,turnover_limpo$industry  )</v>
+      </c>
+      <c r="N3" t="str">
+        <f t="shared" ref="N3:O9" si="4">_xlfn.CONCAT("CramerV( turnover_limpo$",$F$1,",","turnover_limpo$",A3, ")")</f>
+        <v>CramerV( turnover_limpo$coach  ,turnover_limpo$industry  )</v>
+      </c>
+      <c r="O3" t="str">
+        <f t="shared" ref="O3:O9" si="5">_xlfn.CONCAT("CramerV( turnover_limpo$",$G$1,",","turnover_limpo$",A3, ")")</f>
+        <v>CramerV( turnover_limpo$head_gender  ,turnover_limpo$industry  )</v>
+      </c>
+      <c r="P3" t="str">
+        <f t="shared" ref="P3:P9" si="6">_xlfn.CONCAT("CramerV( turnover_limpo$",$H$1,",","turnover_limpo$",A3, ")")</f>
+        <v>CramerV( turnover_limpo$greywage  ,turnover_limpo$industry  )</v>
+      </c>
+      <c r="Q3" t="str">
+        <f t="shared" ref="Q3:Q9" si="7">_xlfn.CONCAT("CramerV( turnover_limpo$",$I$1,",","turnover_limpo$",A3, ")")</f>
+        <v>CramerV( turnover_limpo$way  ,turnover_limpo$industry  )</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="7">
+        <v>0.49558930000000001</v>
+      </c>
+      <c r="C4" s="7">
+        <v>0.23831939999999999</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="7">
+        <v>0.19441079999999999</v>
+      </c>
+      <c r="F4" s="12"/>
+      <c r="J4" t="str">
+        <f t="shared" si="0"/>
+        <v>CramerV( turnover_limpo$gender  ,turnover_limpo$profession  )</v>
+      </c>
+      <c r="K4" t="str">
+        <f t="shared" si="1"/>
+        <v>CramerV( turnover_limpo$industry  ,turnover_limpo$profession  )</v>
+      </c>
+      <c r="L4" t="str">
+        <f t="shared" si="2"/>
+        <v>CramerV( turnover_limpo$profession  ,turnover_limpo$profession  )</v>
+      </c>
+      <c r="M4" t="str">
+        <f t="shared" si="3"/>
+        <v>CramerV( turnover_limpo$traffic  ,turnover_limpo$profession  )</v>
+      </c>
+      <c r="N4" t="str">
+        <f t="shared" si="4"/>
+        <v>CramerV( turnover_limpo$coach  ,turnover_limpo$profession  )</v>
+      </c>
+      <c r="O4" t="str">
+        <f t="shared" si="5"/>
+        <v>CramerV( turnover_limpo$head_gender  ,turnover_limpo$profession  )</v>
+      </c>
+      <c r="P4" t="str">
+        <f t="shared" si="6"/>
+        <v>CramerV( turnover_limpo$greywage  ,turnover_limpo$profession  )</v>
+      </c>
+      <c r="Q4" t="str">
+        <f t="shared" si="7"/>
+        <v>CramerV( turnover_limpo$way  ,turnover_limpo$profession  )</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="7">
+        <v>0.1568532</v>
+      </c>
+      <c r="C5" s="7">
+        <v>0.17210690000000001</v>
+      </c>
+      <c r="D5" s="7">
+        <v>0.19441079999999999</v>
+      </c>
+      <c r="E5" s="7">
+        <v>1</v>
+      </c>
+      <c r="J5" t="str">
+        <f t="shared" si="0"/>
+        <v>CramerV( turnover_limpo$gender  ,turnover_limpo$traffic  )</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="1"/>
+        <v>CramerV( turnover_limpo$industry  ,turnover_limpo$traffic  )</v>
+      </c>
+      <c r="L5" t="str">
+        <f t="shared" si="2"/>
+        <v>CramerV( turnover_limpo$profession  ,turnover_limpo$traffic  )</v>
+      </c>
+      <c r="M5" t="str">
+        <f t="shared" si="3"/>
+        <v>CramerV( turnover_limpo$traffic  ,turnover_limpo$traffic  )</v>
+      </c>
+      <c r="N5" t="str">
+        <f t="shared" si="4"/>
+        <v>CramerV( turnover_limpo$coach  ,turnover_limpo$traffic  )</v>
+      </c>
+      <c r="O5" t="str">
+        <f t="shared" si="5"/>
+        <v>CramerV( turnover_limpo$head_gender  ,turnover_limpo$traffic  )</v>
+      </c>
+      <c r="P5" t="str">
+        <f t="shared" si="6"/>
+        <v>CramerV( turnover_limpo$greywage  ,turnover_limpo$traffic  )</v>
+      </c>
+      <c r="Q5" t="str">
+        <f t="shared" si="7"/>
+        <v>CramerV( turnover_limpo$way  ,turnover_limpo$traffic  )</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="7">
+        <v>7.7273809999999998E-2</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0.14740909999999999</v>
+      </c>
+      <c r="D6" s="7">
+        <v>0.1213484</v>
+      </c>
+      <c r="E6" s="7">
+        <v>0.1125463</v>
+      </c>
+      <c r="J6" t="str">
+        <f t="shared" si="0"/>
+        <v>CramerV( turnover_limpo$gender  ,turnover_limpo$coach  )</v>
+      </c>
+      <c r="K6" t="str">
+        <f t="shared" si="1"/>
+        <v>CramerV( turnover_limpo$industry  ,turnover_limpo$coach  )</v>
+      </c>
+      <c r="L6" t="str">
+        <f t="shared" si="2"/>
+        <v>CramerV( turnover_limpo$profession  ,turnover_limpo$coach  )</v>
+      </c>
+      <c r="M6" t="str">
+        <f t="shared" si="3"/>
+        <v>CramerV( turnover_limpo$traffic  ,turnover_limpo$coach  )</v>
+      </c>
+      <c r="N6" t="str">
+        <f t="shared" si="4"/>
+        <v>CramerV( turnover_limpo$coach  ,turnover_limpo$coach  )</v>
+      </c>
+      <c r="O6" t="str">
+        <f t="shared" si="5"/>
+        <v>CramerV( turnover_limpo$head_gender  ,turnover_limpo$coach  )</v>
+      </c>
+      <c r="P6" t="str">
+        <f t="shared" si="6"/>
+        <v>CramerV( turnover_limpo$greywage  ,turnover_limpo$coach  )</v>
+      </c>
+      <c r="Q6" t="str">
+        <f t="shared" si="7"/>
+        <v>CramerV( turnover_limpo$way  ,turnover_limpo$coach  )</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="7">
+        <v>0.21130489999999999</v>
+      </c>
+      <c r="C7" s="7">
+        <v>0.2445774</v>
+      </c>
+      <c r="D7" s="7">
+        <v>0.33763860000000001</v>
+      </c>
+      <c r="E7" s="7">
+        <v>0.1748479</v>
+      </c>
+      <c r="J7" t="str">
+        <f t="shared" si="0"/>
+        <v>CramerV( turnover_limpo$gender  ,turnover_limpo$head_gender  )</v>
+      </c>
+      <c r="K7" t="str">
+        <f t="shared" si="1"/>
+        <v>CramerV( turnover_limpo$industry  ,turnover_limpo$head_gender  )</v>
+      </c>
+      <c r="L7" t="str">
+        <f t="shared" si="2"/>
+        <v>CramerV( turnover_limpo$profession  ,turnover_limpo$head_gender  )</v>
+      </c>
+      <c r="M7" t="str">
+        <f t="shared" si="3"/>
+        <v>CramerV( turnover_limpo$traffic  ,turnover_limpo$head_gender  )</v>
+      </c>
+      <c r="N7" t="str">
+        <f t="shared" si="4"/>
+        <v>CramerV( turnover_limpo$coach  ,turnover_limpo$head_gender  )</v>
+      </c>
+      <c r="O7" t="str">
+        <f t="shared" si="5"/>
+        <v>CramerV( turnover_limpo$head_gender  ,turnover_limpo$head_gender  )</v>
+      </c>
+      <c r="P7" t="str">
+        <f t="shared" si="6"/>
+        <v>CramerV( turnover_limpo$greywage  ,turnover_limpo$head_gender  )</v>
+      </c>
+      <c r="Q7" t="str">
+        <f t="shared" si="7"/>
+        <v>CramerV( turnover_limpo$way  ,turnover_limpo$head_gender  )</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="7">
+        <v>1.9874380000000001E-2</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0.15171999999999999</v>
+      </c>
+      <c r="D8" s="7">
+        <v>0.16158890000000001</v>
+      </c>
+      <c r="E8" s="7">
+        <v>0.10699740000000001</v>
+      </c>
+      <c r="J8" t="str">
+        <f t="shared" si="0"/>
+        <v>CramerV( turnover_limpo$gender  ,turnover_limpo$greywage  )</v>
+      </c>
+      <c r="K8" t="str">
+        <f t="shared" si="1"/>
+        <v>CramerV( turnover_limpo$industry  ,turnover_limpo$greywage  )</v>
+      </c>
+      <c r="L8" t="str">
+        <f t="shared" si="2"/>
+        <v>CramerV( turnover_limpo$profession  ,turnover_limpo$greywage  )</v>
+      </c>
+      <c r="M8" t="str">
+        <f t="shared" si="3"/>
+        <v>CramerV( turnover_limpo$traffic  ,turnover_limpo$greywage  )</v>
+      </c>
+      <c r="N8" t="str">
+        <f t="shared" si="4"/>
+        <v>CramerV( turnover_limpo$coach  ,turnover_limpo$greywage  )</v>
+      </c>
+      <c r="O8" t="str">
+        <f t="shared" si="5"/>
+        <v>CramerV( turnover_limpo$head_gender  ,turnover_limpo$greywage  )</v>
+      </c>
+      <c r="P8" t="str">
+        <f t="shared" si="6"/>
+        <v>CramerV( turnover_limpo$greywage  ,turnover_limpo$greywage  )</v>
+      </c>
+      <c r="Q8" t="str">
+        <f t="shared" si="7"/>
+        <v>CramerV( turnover_limpo$way  ,turnover_limpo$greywage  )</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="7">
+        <v>0.12719040000000001</v>
+      </c>
+      <c r="C9" s="7">
+        <v>0.20484140000000001</v>
+      </c>
+      <c r="D9" s="7">
+        <v>0.17025589999999999</v>
+      </c>
+      <c r="E9" s="7">
+        <v>0.22651840000000001</v>
+      </c>
+      <c r="J9" t="str">
+        <f t="shared" si="0"/>
+        <v>CramerV( turnover_limpo$gender  ,turnover_limpo$way  )</v>
+      </c>
+      <c r="K9" t="str">
+        <f t="shared" si="1"/>
+        <v>CramerV( turnover_limpo$industry  ,turnover_limpo$way  )</v>
+      </c>
+      <c r="L9" t="str">
+        <f t="shared" si="2"/>
+        <v>CramerV( turnover_limpo$profession  ,turnover_limpo$way  )</v>
+      </c>
+      <c r="M9" t="str">
+        <f t="shared" si="3"/>
+        <v>CramerV( turnover_limpo$traffic  ,turnover_limpo$way  )</v>
+      </c>
+      <c r="N9" t="str">
+        <f t="shared" si="4"/>
+        <v>CramerV( turnover_limpo$coach  ,turnover_limpo$way  )</v>
+      </c>
+      <c r="O9" t="str">
+        <f t="shared" si="5"/>
+        <v>CramerV( turnover_limpo$head_gender  ,turnover_limpo$way  )</v>
+      </c>
+      <c r="P9" t="str">
+        <f t="shared" si="6"/>
+        <v>CramerV( turnover_limpo$greywage  ,turnover_limpo$way  )</v>
+      </c>
+      <c r="Q9" t="str">
+        <f t="shared" si="7"/>
+        <v>CramerV( turnover_limpo$way  ,turnover_limpo$way  )</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D81FAF8-3097-4312-A544-9A64701A1E63}">
   <dimension ref="A1:B15"/>
@@ -3353,22 +3847,22 @@
       <c r="E1" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="11"/>
-      <c r="T1" s="11"/>
-      <c r="U1" s="11"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -3546,22 +4040,22 @@
       </c>
     </row>
     <row r="20" spans="8:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10"/>
-      <c r="O20" s="10"/>
-      <c r="P20" s="10"/>
-      <c r="Q20" s="10"/>
-      <c r="R20" s="10"/>
-      <c r="S20" s="10"/>
-      <c r="T20" s="10"/>
-      <c r="U20" s="10"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="11"/>
+      <c r="N20" s="11"/>
+      <c r="O20" s="11"/>
+      <c r="P20" s="11"/>
+      <c r="Q20" s="11"/>
+      <c r="R20" s="11"/>
+      <c r="S20" s="11"/>
+      <c r="T20" s="11"/>
+      <c r="U20" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>